<commit_message>
feat: implement Day 4 Perception and Body Orientation engine
- Added orientation support to PostGIS schema and Pydantic validation.
- Developed OrientationEngine to extract tactical heading from YOLOv11-OBB.
- Expanded FastAPI Ingestion Server to handle orientation-aware tracking streams.
- Verified end-to-end heading ingestion with live demo and database query.
</commit_message>
<xml_diff>
--- a/AI Sprint_ Football Analytics Plan.xlsx
+++ b/AI Sprint_ Football Analytics Plan.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Sprint Plan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Master Sprint Plan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -563,7 +563,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -607,7 +607,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -629,7 +629,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">

</xml_diff>